<commit_message>
style: move ACH to a separate prominent card
</commit_message>
<xml_diff>
--- a/Data Siswa/Dandi.xlsx
+++ b/Data Siswa/Dandi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Rupa-Rupa\DashboardTim\Data Siswa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7F27719-FAF1-45A4-9BAF-34B1F95598FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7659AF-D63D-42AE-B089-15B047DF8566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{AFE1E578-4FF8-4474-9732-22FF9E651C93}"/>
   </bookViews>
@@ -455,7 +455,7 @@
     <t>Referral</t>
   </si>
   <si>
-    <t>DANDI</t>
+    <t>Irfandi Nyondri</t>
   </si>
 </sst>
 </file>
@@ -511,7 +511,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -530,9 +530,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="15" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1680,7 +1677,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
         <v>60</v>
       </c>
@@ -1696,11 +1693,11 @@
       <c r="E41" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F41" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F41" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
         <v>61</v>
       </c>
@@ -1716,11 +1713,11 @@
       <c r="E42" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F42" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F42" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
         <v>62</v>
       </c>
@@ -1736,11 +1733,11 @@
       <c r="E43" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F43" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F43" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
         <v>63</v>
       </c>
@@ -1756,11 +1753,11 @@
       <c r="E44" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F44" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F44" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A45" s="5" t="s">
         <v>64</v>
       </c>
@@ -1776,11 +1773,11 @@
       <c r="E45" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F45" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F45" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
         <v>65</v>
       </c>
@@ -1796,11 +1793,11 @@
       <c r="E46" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F46" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F46" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
         <v>66</v>
       </c>
@@ -1816,11 +1813,11 @@
       <c r="E47" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F47" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F47" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
         <v>68</v>
       </c>
@@ -1836,11 +1833,11 @@
       <c r="E48" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F48" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F48" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A49" s="5" t="s">
         <v>69</v>
       </c>
@@ -1856,11 +1853,11 @@
       <c r="E49" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F49" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F49" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
         <v>70</v>
       </c>
@@ -1876,11 +1873,11 @@
       <c r="E50" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F50" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F50" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A51" s="5" t="s">
         <v>71</v>
       </c>
@@ -1896,11 +1893,11 @@
       <c r="E51" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F51" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F51" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
         <v>73</v>
       </c>
@@ -1916,11 +1913,11 @@
       <c r="E52" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F52" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F52" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>74</v>
       </c>
@@ -1936,11 +1933,11 @@
       <c r="E53" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F53" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F53" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
         <v>75</v>
       </c>
@@ -1956,11 +1953,11 @@
       <c r="E54" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F54" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F54" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>77</v>
       </c>
@@ -1976,11 +1973,11 @@
       <c r="E55" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F55" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F55" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
         <v>78</v>
       </c>
@@ -1996,11 +1993,11 @@
       <c r="E56" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F56" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F56" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>79</v>
       </c>
@@ -2016,11 +2013,11 @@
       <c r="E57" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F57" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="F57" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="16" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>80</v>
       </c>
@@ -2036,7 +2033,7 @@
       <c r="E58" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F58" s="10" t="s">
+      <c r="F58" s="9" t="s">
         <v>139</v>
       </c>
     </row>

</xml_diff>